<commit_message>
Tighten healthcare corpus semantic review
</commit_message>
<xml_diff>
--- a/clients/healthcare-demo-new/19-template-instantiation-source-corpus/01-template-workbooks/HC_RELATIONSHIP_DICTIONARY.xlsx
+++ b/clients/healthcare-demo-new/19-template-instantiation-source-corpus/01-template-workbooks/HC_RELATIONSHIP_DICTIONARY.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Types" sheetId="1" r:id="R336ba4b88a0742ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Samples" sheetId="2" r:id="Rf255d4c2a62448be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Types" sheetId="1" r:id="R3d6a3633c6644f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Samples" sheetId="2" r:id="R491c7b12cc8046b9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>